<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-18 20:53 UTC
</commit_message>
<xml_diff>
--- a/data/50001555 - ZITRON COLOMBIA ARIS MINING SEGOVIA.xlsx
+++ b/data/50001555 - ZITRON COLOMBIA ARIS MINING SEGOVIA.xlsx
@@ -3448,7 +3448,7 @@
       </c>
       <c r="C27" s="10"/>
       <c r="D27" s="9">
-        <v>46172.18357490741</v>
+        <v>46191.85438790509</v>
       </c>
       <c r="E27" s="10" t="s">
         <v>113</v>
@@ -3629,7 +3629,7 @@
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="5">
-        <v>46169.87942172454</v>
+        <v>46191.85401509259</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>122</v>

</xml_diff>